<commit_message>
V2 dataschema and NHANES dpes
V2 dataschema and NHANES dpes with "months of follow-up" variable
</commit_message>
<xml_diff>
--- a/linkage/dataschema_linkage_mortality.xlsx
+++ b/linkage/dataschema_linkage_mortality.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Computer\twey working files\ProPASS\DataSchemas\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\twey\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FEB80819-DFEA-431C-861E-0D8D9A4E981D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B8D993CE-622B-4AE4-91F7-507EEA134481}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19090" yWindow="1840" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{DBFF5EF0-97C7-4AC5-AB4B-7CA3D94442ED}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DBFF5EF0-97C7-4AC5-AB4B-7CA3D94442ED}"/>
   </bookViews>
   <sheets>
     <sheet name="Variables" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="97">
   <si>
     <t>index</t>
   </si>
@@ -313,6 +313,21 @@
   </si>
   <si>
     <t>dth_cancer_nhanes</t>
+  </si>
+  <si>
+    <t>months</t>
+  </si>
+  <si>
+    <t>dth_months_followup</t>
+  </si>
+  <si>
+    <t>Months of follow-up</t>
+  </si>
+  <si>
+    <t>If this is calculated from difference between two dates, round to nearest whole month.</t>
+  </si>
+  <si>
+    <t>Number of months of participant follow-up from baseline</t>
   </si>
 </sst>
 </file>
@@ -348,18 +363,12 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -381,23 +390,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -733,7 +741,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B57A8CD-7ECD-4C2F-A433-3DF4AB5DDFFE}">
-  <dimension ref="A1:N22"/>
+  <dimension ref="A1:N23"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6" bestFit="1" customWidth="1"/>
@@ -745,10 +753,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
@@ -827,13 +835,13 @@
       <c r="C3" t="s">
         <v>58</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" t="s">
         <v>59</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" t="s">
         <v>60</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="F3" t="s">
         <v>61</v>
       </c>
       <c r="G3" t="s">
@@ -856,13 +864,13 @@
       <c r="C4" t="s">
         <v>58</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" t="s">
         <v>64</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="E4" t="s">
         <v>65</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="F4" t="s">
         <v>66</v>
       </c>
       <c r="G4" t="s">
@@ -885,13 +893,13 @@
       <c r="C5" t="s">
         <v>58</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="D5" t="s">
         <v>69</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="E5" t="s">
         <v>70</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="F5" t="s">
         <v>71</v>
       </c>
       <c r="G5" t="s">
@@ -911,13 +919,13 @@
       <c r="C6" t="s">
         <v>58</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" t="s">
         <v>72</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="E6" t="s">
         <v>73</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="F6" t="s">
         <v>73</v>
       </c>
       <c r="G6" t="s">
@@ -946,13 +954,13 @@
       <c r="C7" t="s">
         <v>58</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" t="s">
         <v>77</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" t="s">
         <v>78</v>
       </c>
-      <c r="F7" s="7" t="s">
+      <c r="F7" t="s">
         <v>78</v>
       </c>
       <c r="G7" t="s">
@@ -981,13 +989,13 @@
       <c r="C8" t="s">
         <v>58</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" t="s">
         <v>79</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" t="s">
         <v>80</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="F8" t="s">
         <v>81</v>
       </c>
       <c r="G8" t="s">
@@ -1013,13 +1021,13 @@
       <c r="C9" t="s">
         <v>58</v>
       </c>
-      <c r="D9" s="1" t="s">
+      <c r="D9" t="s">
         <v>17</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="E9" t="s">
         <v>86</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="F9" t="s">
         <v>86</v>
       </c>
       <c r="G9" t="s">
@@ -1045,13 +1053,13 @@
       <c r="C10" t="s">
         <v>58</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="D10" t="s">
         <v>16</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="E10" t="s">
         <v>87</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="F10" t="s">
         <v>87</v>
       </c>
       <c r="G10" t="s">
@@ -1077,13 +1085,13 @@
       <c r="C11" t="s">
         <v>58</v>
       </c>
-      <c r="D11" s="1" t="s">
+      <c r="D11" t="s">
         <v>15</v>
       </c>
-      <c r="E11" s="1" t="s">
+      <c r="E11" t="s">
         <v>88</v>
       </c>
-      <c r="F11" s="1" t="s">
+      <c r="F11" t="s">
         <v>88</v>
       </c>
       <c r="G11" t="s">
@@ -1109,23 +1117,29 @@
       <c r="C12" t="s">
         <v>58</v>
       </c>
-      <c r="D12" t="s">
-        <v>56</v>
-      </c>
-      <c r="E12" t="s">
-        <v>57</v>
-      </c>
-      <c r="F12" t="s">
-        <v>57</v>
-      </c>
-      <c r="G12" t="s">
-        <v>31</v>
+      <c r="D12" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H12" s="6" t="s">
+        <v>92</v>
       </c>
       <c r="J12" t="s">
         <v>82</v>
       </c>
       <c r="L12" t="s">
         <v>85</v>
+      </c>
+      <c r="M12" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
@@ -1139,16 +1153,16 @@
         <v>58</v>
       </c>
       <c r="D13" t="s">
-        <v>39</v>
+        <v>56</v>
       </c>
       <c r="E13" t="s">
-        <v>18</v>
+        <v>57</v>
       </c>
       <c r="F13" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="G13" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J13" t="s">
         <v>82</v>
@@ -1167,14 +1181,14 @@
       <c r="C14" t="s">
         <v>58</v>
       </c>
-      <c r="D14" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="E14" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="F14" s="7" t="s">
-        <v>90</v>
+      <c r="D14" t="s">
+        <v>39</v>
+      </c>
+      <c r="E14" t="s">
+        <v>18</v>
+      </c>
+      <c r="F14" t="s">
+        <v>48</v>
       </c>
       <c r="G14" t="s">
         <v>32</v>
@@ -1197,13 +1211,13 @@
         <v>58</v>
       </c>
       <c r="D15" t="s">
-        <v>40</v>
+        <v>91</v>
       </c>
       <c r="E15" t="s">
-        <v>19</v>
+        <v>84</v>
       </c>
       <c r="F15" t="s">
-        <v>49</v>
+        <v>90</v>
       </c>
       <c r="G15" t="s">
         <v>32</v>
@@ -1226,13 +1240,13 @@
         <v>58</v>
       </c>
       <c r="D16" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E16" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F16" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G16" t="s">
         <v>32</v>
@@ -1255,13 +1269,13 @@
         <v>58</v>
       </c>
       <c r="D17" t="s">
-        <v>21</v>
+        <v>41</v>
       </c>
       <c r="E17" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F17" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G17" t="s">
         <v>32</v>
@@ -1284,13 +1298,13 @@
         <v>58</v>
       </c>
       <c r="D18" t="s">
-        <v>42</v>
+        <v>21</v>
       </c>
       <c r="E18" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F18" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G18" t="s">
         <v>32</v>
@@ -1313,13 +1327,13 @@
         <v>58</v>
       </c>
       <c r="D19" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E19" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F19" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G19" t="s">
         <v>32</v>
@@ -1342,13 +1356,13 @@
         <v>58</v>
       </c>
       <c r="D20" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E20" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F20" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G20" t="s">
         <v>32</v>
@@ -1371,13 +1385,13 @@
         <v>58</v>
       </c>
       <c r="D21" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E21" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F21" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="G21" t="s">
         <v>32</v>
@@ -1400,13 +1414,13 @@
         <v>58</v>
       </c>
       <c r="D22" t="s">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="E22" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="F22" t="s">
-        <v>28</v>
+        <v>55</v>
       </c>
       <c r="G22" t="s">
         <v>32</v>
@@ -1415,6 +1429,35 @@
         <v>82</v>
       </c>
       <c r="L22" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" t="s">
+        <v>29</v>
+      </c>
+      <c r="C23" t="s">
+        <v>58</v>
+      </c>
+      <c r="D23" t="s">
+        <v>27</v>
+      </c>
+      <c r="E23" t="s">
+        <v>28</v>
+      </c>
+      <c r="F23" t="s">
+        <v>28</v>
+      </c>
+      <c r="G23" t="s">
+        <v>32</v>
+      </c>
+      <c r="J23" t="s">
+        <v>82</v>
+      </c>
+      <c r="L23" t="s">
         <v>85</v>
       </c>
     </row>
@@ -1437,22 +1480,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="F1" s="5" t="s">
         <v>14</v>
       </c>
     </row>
@@ -1503,7 +1546,7 @@
       <c r="B4" t="s">
         <v>58</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" t="s">
         <v>91</v>
       </c>
       <c r="D4">
@@ -1523,7 +1566,7 @@
       <c r="B5" t="s">
         <v>58</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" t="s">
         <v>91</v>
       </c>
       <c r="D5">

</xml_diff>

<commit_message>
Change DS label:en to label
</commit_message>
<xml_diff>
--- a/linkage/dataschema_linkage_mortality.xlsx
+++ b/linkage/dataschema_linkage_mortality.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\twey\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BAB5FE9-4A37-4547-B0F9-A6EF8AC54F5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C164C70-06BE-428A-B6B4-7EC45F2EF1A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DBFF5EF0-97C7-4AC5-AB4B-7CA3D94442ED}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="96">
   <si>
     <t>index</t>
   </si>
@@ -49,9 +49,6 @@
   </si>
   <si>
     <t>name</t>
-  </si>
-  <si>
-    <t>label:en</t>
   </si>
   <si>
     <t>valueType</t>
@@ -772,34 +769,34 @@
         <v>3</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="J1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="K1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="L1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="M1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="N1" s="3" t="s">
         <v>11</v>
-      </c>
-      <c r="N1" s="3" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
@@ -807,28 +804,28 @@
         <v>1</v>
       </c>
       <c r="B2" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="E2" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C2" s="6" t="s">
-        <v>95</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="E2" s="6" t="s">
+      <c r="F2" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="G2" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="F2" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="G2" s="6" t="s">
-        <v>31</v>
-      </c>
       <c r="J2" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="L2" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
@@ -836,28 +833,28 @@
         <v>2</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D3" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="E3" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="F3" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="G3" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="J3" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="G3" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="J3" s="6" t="s">
+      <c r="M3" s="6" t="s">
         <v>61</v>
-      </c>
-      <c r="M3" s="6" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
@@ -865,28 +862,28 @@
         <v>3</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D4" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="E4" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="F4" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="G4" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="J4" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="G4" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="J4" s="6" t="s">
+      <c r="M4" s="6" t="s">
         <v>66</v>
-      </c>
-      <c r="M4" s="6" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
@@ -894,25 +891,25 @@
         <v>4</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D5" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="E5" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="F5" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="F5" s="6" t="s">
-        <v>70</v>
-      </c>
       <c r="G5" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="J5" s="6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
@@ -920,34 +917,34 @@
         <v>5</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D6" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="E6" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="F6" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="I6" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="J6" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="F6" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="G6" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="I6" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="J6" s="6" t="s">
+      <c r="K6" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="K6" s="6" t="s">
+      <c r="M6" s="6" t="s">
         <v>74</v>
-      </c>
-      <c r="M6" s="6" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
@@ -955,34 +952,34 @@
         <v>6</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D7" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="E7" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="E7" s="6" t="s">
-        <v>77</v>
-      </c>
       <c r="F7" s="6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="J7" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="K7" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="K7" s="6" t="s">
+      <c r="M7" s="6" t="s">
         <v>74</v>
-      </c>
-      <c r="M7" s="6" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
@@ -990,34 +987,34 @@
         <v>7</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C8" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="D8" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="D8" s="7" t="s">
-        <v>96</v>
-      </c>
       <c r="E8" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="H8" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="J8" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="L8" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="M8" s="6" t="s">
         <v>92</v>
-      </c>
-      <c r="F8" s="7" t="s">
-        <v>94</v>
-      </c>
-      <c r="G8" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="H8" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="J8" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="L8" s="6" t="s">
-        <v>84</v>
-      </c>
-      <c r="M8" s="6" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
@@ -1025,31 +1022,31 @@
         <v>8</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D9" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="E9" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="F9" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="F9" s="6" t="s">
+      <c r="G9" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="J9" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="G9" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="J9" s="6" t="s">
-        <v>81</v>
-      </c>
       <c r="K9" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="L9" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
@@ -1057,31 +1054,31 @@
         <v>9</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G10" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="I10" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="I10" s="6" t="s">
-        <v>33</v>
-      </c>
       <c r="J10" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="L10" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
@@ -1089,31 +1086,31 @@
         <v>10</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="I11" s="6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="J11" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="L11" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
@@ -1121,31 +1118,31 @@
         <v>11</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="I12" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="J12" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="L12" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
@@ -1153,28 +1150,28 @@
         <v>12</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D13" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="E13" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="E13" s="6" t="s">
-        <v>57</v>
-      </c>
       <c r="F13" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="J13" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="L13" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
@@ -1182,28 +1179,28 @@
         <v>13</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J14" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="L14" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
@@ -1211,28 +1208,28 @@
         <v>14</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E15" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="J15" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="L15" s="6" t="s">
         <v>83</v>
-      </c>
-      <c r="F15" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="G15" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="J15" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="L15" s="6" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
@@ -1240,28 +1237,28 @@
         <v>15</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J16" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="L16" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.25">
@@ -1269,28 +1266,28 @@
         <v>16</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J17" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="L17" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.25">
@@ -1298,28 +1295,28 @@
         <v>17</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D18" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="E18" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="E18" s="6" t="s">
-        <v>22</v>
-      </c>
       <c r="F18" s="6" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G18" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J18" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="L18" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.25">
@@ -1327,28 +1324,28 @@
         <v>18</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J19" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="L19" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.25">
@@ -1356,28 +1353,28 @@
         <v>19</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G20" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J20" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="L20" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">
@@ -1385,28 +1382,28 @@
         <v>20</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G21" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J21" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="L21" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.25">
@@ -1414,28 +1411,28 @@
         <v>21</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="G22" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J22" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="L22" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.25">
@@ -1443,28 +1440,28 @@
         <v>22</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D23" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="E23" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="E23" s="6" t="s">
-        <v>28</v>
-      </c>
       <c r="F23" s="6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G23" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J23" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="L23" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
   </sheetData>
@@ -1493,416 +1490,416 @@
         <v>2</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>4</v>
+        <v>87</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D2">
         <v>0</v>
       </c>
       <c r="E2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D3">
         <v>1</v>
       </c>
       <c r="E3" t="s">
+        <v>36</v>
+      </c>
+      <c r="F3" t="s">
         <v>37</v>
-      </c>
-      <c r="F3" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D4">
         <v>0</v>
       </c>
       <c r="E4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B5" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D5">
         <v>1</v>
       </c>
       <c r="E5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F5" t="s">
         <v>37</v>
-      </c>
-      <c r="F5" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D6">
         <v>0</v>
       </c>
       <c r="E6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B7" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D7">
         <v>1</v>
       </c>
       <c r="E7" t="s">
+        <v>36</v>
+      </c>
+      <c r="F7" t="s">
         <v>37</v>
-      </c>
-      <c r="F7" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B8" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D8">
         <v>0</v>
       </c>
       <c r="E8" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B9" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D9">
         <v>1</v>
       </c>
       <c r="E9" t="s">
+        <v>36</v>
+      </c>
+      <c r="F9" t="s">
         <v>37</v>
-      </c>
-      <c r="F9" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B10" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D10">
         <v>0</v>
       </c>
       <c r="E10" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B11" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C11" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D11">
         <v>1</v>
       </c>
       <c r="E11" t="s">
+        <v>36</v>
+      </c>
+      <c r="F11" t="s">
         <v>37</v>
-      </c>
-      <c r="F11" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B12" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C12" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D12">
         <v>0</v>
       </c>
       <c r="E12" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F12" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B13" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C13" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D13">
         <v>1</v>
       </c>
       <c r="E13" t="s">
+        <v>36</v>
+      </c>
+      <c r="F13" t="s">
         <v>37</v>
-      </c>
-      <c r="F13" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B14" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D14">
         <v>0</v>
       </c>
       <c r="E14" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F14" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B15" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D15">
         <v>1</v>
       </c>
       <c r="E15" t="s">
+        <v>36</v>
+      </c>
+      <c r="F15" t="s">
         <v>37</v>
-      </c>
-      <c r="F15" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B16" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C16" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D16">
         <v>0</v>
       </c>
       <c r="E16" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F16" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B17" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C17" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D17">
         <v>1</v>
       </c>
       <c r="E17" t="s">
+        <v>36</v>
+      </c>
+      <c r="F17" t="s">
         <v>37</v>
-      </c>
-      <c r="F17" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B18" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C18" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D18">
         <v>0</v>
       </c>
       <c r="E18" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F18" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B19" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C19" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D19">
         <v>1</v>
       </c>
       <c r="E19" t="s">
+        <v>36</v>
+      </c>
+      <c r="F19" t="s">
         <v>37</v>
-      </c>
-      <c r="F19" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B20" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C20" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D20">
         <v>0</v>
       </c>
       <c r="E20" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F20" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B21" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C21" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D21">
         <v>1</v>
       </c>
       <c r="E21" t="s">
+        <v>36</v>
+      </c>
+      <c r="F21" t="s">
         <v>37</v>
-      </c>
-      <c r="F21" t="s">
-        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>